<commit_message>
Basic Motion Study Added to the Lift
</commit_message>
<xml_diff>
--- a/Phase-A_design/03_lift-cad-dfm/BOM.xlsx
+++ b/Phase-A_design/03_lift-cad-dfm/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ah Shit Here We Go Again\Major Projects\Graduation Project 2027\AGV-Mechanical-Phase\Phase-A_design\03_lift-cad-dfm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C11B5C7A-CD14-41BC-86B3-52EEA2E86F6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A36B5356-F37D-4C33-9F22-1C516C7F2F63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{E39E7D54-E321-4444-97C1-205676E06357}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>RodSBR</t>
   </si>
@@ -61,16 +60,34 @@
   </si>
   <si>
     <t>Item</t>
+  </si>
+  <si>
+    <t>Circlip</t>
+  </si>
+  <si>
+    <t>M5x16</t>
+  </si>
+  <si>
+    <t>M5x12</t>
+  </si>
+  <si>
+    <t>M5 Lock Nuts</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -535,24 +552,36 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
       <c r="D8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
       <c r="D9">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
       <c r="D10">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
       <c r="D11">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -612,6 +641,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>